<commit_message>
feat: add configurable enchantment rolls per lick
Keep EnchantTimes as the saliva-based level multiplier and add EnchantCount for one to ten rolls during a single successful lick. Replace only the reviewed TryLickEnchant call so global enchantment generation and one-lick eligibility remain unchanged.
</commit_message>
<xml_diff>
--- a/LangConfig/CN.xlsx
+++ b/LangConfig/CN.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -565,15 +565,32 @@
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>EnchantCount</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>每次舔舐附魔次数</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>每次成功舔物品时执行的附魔抽取次数。有效范围为 1 到 10；重复抽中同一附魔时会叠加其等级。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>RequireLickAbility</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>需要艾赫卡托尔的祝福</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>启用后，当前地图必须有角色拥有“艾赫卡托尔的祝福”特质。关闭后由玩家触发相关效果。</t>
         </is>

</xml_diff>